<commit_message>
functional and non-functional requirements v1.0.0
</commit_message>
<xml_diff>
--- a/input/system-requirements/SRV DAK_functional and non-functional requirements.xlsx
+++ b/input/system-requirements/SRV DAK_functional and non-functional requirements.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://greeninkltd-my.sharepoint.com/personal/vfc_greenink_co_uk/Documents/Live Jobs/WHO Health Emergencies/GIP03451/2_Edited files/edit3/work in progress/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="65" documentId="13_ncr:1_{B42C4E21-00CB-504C-93F6-2E5BE549F991}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{6EC93DC2-AE0A-476A-B69C-A92027AA0281}"/>
+  <xr:revisionPtr revIDLastSave="65" documentId="13_ncr:1_{B42C4E21-00CB-504C-93F6-2E5BE549F991}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{9E779A7D-C09F-4111-8054-6FAECCF4221B}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{A364870C-86B3-C147-A494-BA544CC03900}"/>
   </bookViews>
@@ -203,8 +203,8 @@
     <t>The non-functional requirement</t>
   </si>
   <si>
-    <t>https://smart.who.int/dak-srv/v0.9.9/SRV DAK_functional and non-functional requirements.xlsx
-© World Health Organization 2026. Some rights reserved. This work is available under the:</t>
+    <t xml:space="preserve">https://smart.who.int/dak-srv/v1.0.0/SRV DAK_functional and non-functional requirements.xlsx
+© World Health Organization 2026. Some rights reserved. This work is available under the: </t>
   </si>
   <si>
     <t>CC BY-NC-SA 4.0 licence</t>
@@ -4509,7 +4509,7 @@
       <c r="J22" s="17"/>
       <c r="K22" s="17"/>
     </row>
-    <row r="23" spans="1:11" ht="32.25" customHeight="1">
+    <row r="23" spans="1:11" ht="31.5" customHeight="1">
       <c r="A23" s="17"/>
       <c r="B23" s="46" t="s">
         <v>24</v>

</xml_diff>